<commit_message>
Personalkorten: dold 'Lindring'/'Händelsemotstånd' borttagen
Projektchefernas och arbetschefernas kort hade otryckt speldata (lindra politik-, dialog-
och nämndkort med 1/3/5) som inte syntes på korten och aldrig användes av motorn. Beslut
(Niklas): allt som gäller ska stå på korten – kolumnerna tas bort ur kortdata och ur
verktyg/bygg_personal_excel.py.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JCFLjpHxkTTwZndbAW5eBH
</commit_message>
<xml_diff>
--- a/kortdata/L_personal.xlsx
+++ b/kortdata/L_personal.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y19"/>
+  <dimension ref="A1:W19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -550,40 +550,30 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Lindring</t>
+          <t>Nämnd</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>Händelsemotstånd</t>
+          <t>Kvalitet Q</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>Nämnd</t>
+          <t>Hållbarhet H</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>Kvalitet Q</t>
+          <t>Tid T</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>Hållbarhet H</t>
+          <t>Erfarenhet</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>Tid T</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>Erfarenhet</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Antal exemplar</t>
         </is>
@@ -692,17 +682,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="W2" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X2" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y2" s="2" t="n">
+      <c r="W2" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -809,17 +789,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="W3" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X3" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y3" s="2" t="n">
+      <c r="W3" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -926,17 +896,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="W4" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X4" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y4" s="2" t="n">
+      <c r="W4" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1043,17 +1003,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="W5" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X5" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y5" s="2" t="n">
+      <c r="W5" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1160,17 +1110,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="W6" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X6" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y6" s="2" t="n">
+      <c r="W6" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1277,17 +1217,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="W7" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X7" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y7" s="2" t="n">
+      <c r="W7" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1396,17 +1326,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="W8" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X8" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y8" s="2" t="n">
+      <c r="W8" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1513,17 +1433,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="W9" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X9" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y9" s="2" t="n">
+      <c r="W9" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1630,17 +1540,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="W10" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X10" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y10" s="2" t="n">
+      <c r="W10" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1747,17 +1647,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="W11" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X11" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y11" s="2" t="n">
+      <c r="W11" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1864,17 +1754,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="W12" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X12" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y12" s="2" t="n">
+      <c r="W12" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1981,17 +1861,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="W13" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X13" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y13" s="2" t="n">
+      <c r="W13" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2098,17 +1968,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="W14" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X14" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y14" s="2" t="n">
+      <c r="W14" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2215,17 +2075,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="W15" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X15" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y15" s="2" t="n">
+      <c r="W15" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2332,17 +2182,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="W16" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X16" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y16" s="2" t="n">
+      <c r="W16" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2449,17 +2289,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="W17" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X17" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y17" s="2" t="n">
+      <c r="W17" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2566,17 +2396,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="W18" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X18" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y18" s="2" t="n">
+      <c r="W18" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2685,17 +2505,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="W19" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X19" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y19" s="2" t="n">
+      <c r="W19" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3850,7 +3660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4258,12 +4068,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Lindring</t>
+          <t>Nämnd</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Lindring</t>
+          <t>Nämnd</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -4280,12 +4090,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Händelsemotstånd</t>
+          <t>Kvalitet Q</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Händelsemotstand</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -4302,12 +4112,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Nämnd</t>
+          <t>Hållbarhet H</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Nämnd</t>
+          <t>H</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -4324,12 +4134,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Kvalitet Q</t>
+          <t>Tid T</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -4346,12 +4156,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Hållbarhet H</t>
+          <t>Erfarenhet</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>Erfarenhet</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -4368,12 +4178,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Tid T</t>
+          <t>Antal exemplar</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -4382,50 +4192,6 @@
         </is>
       </c>
       <c r="D24" t="inlineStr">
-        <is>
-          <t>Ej tryckt — '-' på alla ledningskort</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Erfarenhet</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Erfarenhet</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Ej tryckt — '-' på alla ledningskort</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Antal exemplar</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
         <is>
           <t>Antal tryckta kort per spel (exemplar_map: 1)</t>
         </is>

</xml_diff>